<commit_message>
update size of app view
</commit_message>
<xml_diff>
--- a/cn-med-kg/medicine_dataset.xlsx
+++ b/cn-med-kg/medicine_dataset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Chinese_Medicine\cn-med-kg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2742809D-9C4D-409F-906D-D37BE966E1A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7ACA7A5-B901-4375-B8C5-CA5E611F6B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FCBB9041-7F32-418A-9A6B-AB2AB6A56C91}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FCBB9041-7F32-418A-9A6B-AB2AB6A56C91}"/>
   </bookViews>
   <sheets>
     <sheet name="1-namelist" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="219">
   <si>
     <t>药品名称</t>
   </si>
@@ -609,6 +609,93 @@
   </si>
   <si>
     <t>缓解咽部疼痛不适</t>
+  </si>
+  <si>
+    <t>丹七片</t>
+  </si>
+  <si>
+    <t>m000010</t>
+  </si>
+  <si>
+    <t>Danqi Pian</t>
+  </si>
+  <si>
+    <t>北京同仁堂科技发展股份有限公司制药厂</t>
+  </si>
+  <si>
+    <t>国药准字Z11020471</t>
+  </si>
+  <si>
+    <t>丹参</t>
+  </si>
+  <si>
+    <t>活血化瘀</t>
+  </si>
+  <si>
+    <t>血瘀气滞</t>
+  </si>
+  <si>
+    <t>心胸痹痛</t>
+  </si>
+  <si>
+    <t>眩晕头痛</t>
+  </si>
+  <si>
+    <t>经期腹痛</t>
+  </si>
+  <si>
+    <t>山药薏米莲子粥</t>
+  </si>
+  <si>
+    <t>m000011</t>
+  </si>
+  <si>
+    <t>粥之养</t>
+  </si>
+  <si>
+    <t>Zhou Zhi Yang</t>
+  </si>
+  <si>
+    <t>山东杰格郎食品有限公司</t>
+  </si>
+  <si>
+    <t>山东省临沂市沂水县崔家峪镇兖石路7号</t>
+  </si>
+  <si>
+    <t>4000096667</t>
+  </si>
+  <si>
+    <t>Q/JGL0001S</t>
+  </si>
+  <si>
+    <t>大麦仁</t>
+  </si>
+  <si>
+    <t>糯米</t>
+  </si>
+  <si>
+    <t>海藻糖</t>
+  </si>
+  <si>
+    <t>赤小豆</t>
+  </si>
+  <si>
+    <t>白扁豆</t>
+  </si>
+  <si>
+    <t>薏米</t>
+  </si>
+  <si>
+    <t>山药</t>
+  </si>
+  <si>
+    <t>芡实</t>
+  </si>
+  <si>
+    <t>莲子</t>
+  </si>
+  <si>
+    <t>枸杞</t>
   </si>
 </sst>
 </file>
@@ -770,7 +857,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -789,29 +876,13 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="36">
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="none">
@@ -1158,6 +1229,21 @@
         <left style="thin">
           <color indexed="64"/>
         </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
         <right style="thin">
           <color indexed="64"/>
         </right>
@@ -1308,6 +1394,7 @@
       </border>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -1413,13 +1500,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2091243D-01EB-417B-A545-8F66A0029A2F}" name="Table2" displayName="Table2" ref="A1:K10" totalsRowShown="0" headerRowDxfId="35" headerRowBorderDxfId="34" tableBorderDxfId="33" totalsRowBorderDxfId="32">
-  <autoFilter ref="A1:K10" xr:uid="{2091243D-01EB-417B-A545-8F66A0029A2F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2091243D-01EB-417B-A545-8F66A0029A2F}" name="Table2" displayName="Table2" ref="A1:K12" totalsRowShown="0" headerRowDxfId="35" headerRowBorderDxfId="34" tableBorderDxfId="33" totalsRowBorderDxfId="32">
+  <autoFilter ref="A1:K12" xr:uid="{2091243D-01EB-417B-A545-8F66A0029A2F}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{70404F4C-EA74-419B-B8F7-C0E749DBA8EF}" name="药品名称" dataDxfId="31"/>
-    <tableColumn id="7" xr3:uid="{A127C5AC-1A8D-4194-B82B-CEA8C46568A9}" name="UID" dataDxfId="30">
-      <calculatedColumnFormula>"m00000" &amp; TEXT(ROW() - ROW(Table2[[#Headers],[UID]]), "0;-0")</calculatedColumnFormula>
-    </tableColumn>
+    <tableColumn id="7" xr3:uid="{A127C5AC-1A8D-4194-B82B-CEA8C46568A9}" name="UID" dataDxfId="30"/>
     <tableColumn id="2" xr3:uid="{745BAE8D-3E74-492D-9F1F-A46F418B7407}" name="品牌" dataDxfId="29"/>
     <tableColumn id="8" xr3:uid="{4568304F-01F3-4E31-A34C-C35C96C88C80}" name="NameEnglish" dataDxfId="28"/>
     <tableColumn id="9" xr3:uid="{8640C111-58A7-4B70-8A2F-6ECA558B9042}" name="BrandEnglish" dataDxfId="27"/>
@@ -1427,42 +1512,42 @@
     <tableColumn id="5" xr3:uid="{76794CF7-5E96-4BA4-A111-0F4FB586AAEB}" name="生产商地址" dataDxfId="25"/>
     <tableColumn id="10" xr3:uid="{835D09B6-5D13-418C-9FB4-33A768C770CA}" name="生产商网址" dataDxfId="24"/>
     <tableColumn id="6" xr3:uid="{098A7009-4AD7-411F-A1F5-1CE1E004D519}" name="生产商电话" dataDxfId="23"/>
-    <tableColumn id="11" xr3:uid="{A8035F40-8DAA-459C-8132-AB84A20FE398}" name="批准文号" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{2B5D44FA-F4F3-4890-8993-4D8C1FD7AA21}" name="执行标准" dataDxfId="22"/>
+    <tableColumn id="11" xr3:uid="{A8035F40-8DAA-459C-8132-AB84A20FE398}" name="批准文号" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{2B5D44FA-F4F3-4890-8993-4D8C1FD7AA21}" name="执行标准" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{14ED46AD-AD3A-4EEB-8896-42FDC45797B6}" name="Table3" displayName="Table3" ref="A1:C97" totalsRowShown="0" headerRowDxfId="21" headerRowBorderDxfId="20" tableBorderDxfId="19" totalsRowBorderDxfId="18">
-  <autoFilter ref="A1:C97" xr:uid="{14ED46AD-AD3A-4EEB-8896-42FDC45797B6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{14ED46AD-AD3A-4EEB-8896-42FDC45797B6}" name="Table3" displayName="Table3" ref="A1:C110" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="19" tableBorderDxfId="18" totalsRowBorderDxfId="17">
+  <autoFilter ref="A1:C110" xr:uid="{14ED46AD-AD3A-4EEB-8896-42FDC45797B6}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{9CBDF56B-3BCD-4FF2-8195-561FA1F4C31A}" name="药品ID" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{77270F8D-0C55-4EBC-B9E0-6E3C41859F9D}" name="成分" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{FC03B7AA-E421-4532-B8E6-ECB424CCAB8A}" name="ComponentEnglish" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{9CBDF56B-3BCD-4FF2-8195-561FA1F4C31A}" name="药品ID" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{77270F8D-0C55-4EBC-B9E0-6E3C41859F9D}" name="成分" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{FC03B7AA-E421-4532-B8E6-ECB424CCAB8A}" name="ComponentEnglish" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CA49AA06-1ABA-4D07-85FE-0008DCD2BD44}" name="Table5" displayName="Table5" ref="A1:B7" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
-  <autoFilter ref="A1:B7" xr:uid="{CA49AA06-1ABA-4D07-85FE-0008DCD2BD44}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CA49AA06-1ABA-4D07-85FE-0008DCD2BD44}" name="Table5" displayName="Table5" ref="A1:B8" totalsRowShown="0" headerRowDxfId="13" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10" totalsRowBorderDxfId="9">
+  <autoFilter ref="A1:B8" xr:uid="{CA49AA06-1ABA-4D07-85FE-0008DCD2BD44}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{B8626E94-0403-419E-8E68-71E33A149F5F}" name="药品ID" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{69B649F7-4B8F-4BD8-8C6B-CA5943FF7F38}" name="功能" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{B8626E94-0403-419E-8E68-71E33A149F5F}" name="药品ID" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{69B649F7-4B8F-4BD8-8C6B-CA5943FF7F38}" name="功能" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{959167B2-548D-49FA-94EE-4B29E8917423}" name="Table4" displayName="Table4" ref="A1:B8" totalsRowShown="0" headerRowDxfId="7" dataDxfId="5" headerRowBorderDxfId="6" tableBorderDxfId="4" totalsRowBorderDxfId="3">
-  <autoFilter ref="A1:B8" xr:uid="{959167B2-548D-49FA-94EE-4B29E8917423}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{959167B2-548D-49FA-94EE-4B29E8917423}" name="Table4" displayName="Table4" ref="A1:B12" totalsRowShown="0" headerRowDxfId="6" dataDxfId="4" headerRowBorderDxfId="5" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+  <autoFilter ref="A1:B12" xr:uid="{959167B2-548D-49FA-94EE-4B29E8917423}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{B3E95E7E-96F3-4FFA-B777-46887DE69A33}" name="药品ID" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{65C8285F-658B-48F3-A03C-C101895E22EF}" name="主治" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{B3E95E7E-96F3-4FFA-B777-46887DE69A33}" name="药品ID" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{65C8285F-658B-48F3-A03C-C101895E22EF}" name="主治" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1785,7 +1870,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26C0E823-9BD2-43CB-A179-B4CF5CB62E6F}">
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
@@ -1840,9 +1925,8 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="10" t="str">
-        <f>"m00000" &amp; TEXT(ROW() - ROW(Table2[[#Headers],[UID]]), "0;-0")</f>
-        <v>m000001</v>
+      <c r="B2" s="10" t="s">
+        <v>77</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>3</v>
@@ -1870,9 +1954,8 @@
       <c r="A3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="10" t="str">
-        <f>"m00000" &amp; TEXT(ROW() - ROW(Table2[[#Headers],[UID]]), "0;-0")</f>
-        <v>m000002</v>
+      <c r="B3" s="10" t="s">
+        <v>78</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>29</v>
@@ -1900,9 +1983,8 @@
       <c r="A4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="10" t="str">
-        <f>"m00000" &amp; TEXT(ROW() - ROW(Table2[[#Headers],[UID]]), "0;-0")</f>
-        <v>m000003</v>
+      <c r="B4" s="10" t="s">
+        <v>79</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>38</v>
@@ -1930,9 +2012,8 @@
       <c r="A5" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B5" s="10" t="str">
-        <f>"m00000" &amp; TEXT(ROW() - ROW(Table2[[#Headers],[UID]]), "0;-0")</f>
-        <v>m000004</v>
+      <c r="B5" s="10" t="s">
+        <v>80</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>72</v>
@@ -1958,9 +2039,8 @@
       <c r="A6" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B6" s="10" t="str">
-        <f>"m00000" &amp; TEXT(ROW() - ROW(Table2[[#Headers],[UID]]), "0;-0")</f>
-        <v>m000005</v>
+      <c r="B6" s="10" t="s">
+        <v>89</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>90</v>
@@ -1986,9 +2066,8 @@
       <c r="A7" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B7" s="7" t="str">
-        <f>"m00000" &amp; TEXT(ROW() - ROW(Table2[[#Headers],[UID]]), "0;-0")</f>
-        <v>m000006</v>
+      <c r="B7" s="7" t="s">
+        <v>107</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>102</v>
@@ -2018,9 +2097,8 @@
       <c r="A8" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="B8" s="7" t="str">
-        <f>"m00000" &amp; TEXT(ROW() - ROW(Table2[[#Headers],[UID]]), "0;-0")</f>
-        <v>m000007</v>
+      <c r="B8" s="7" t="s">
+        <v>143</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>140</v>
@@ -2044,9 +2122,8 @@
       <c r="A9" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="B9" s="7" t="str">
-        <f>"m00000" &amp; TEXT(ROW() - ROW(Table2[[#Headers],[UID]]), "0;-0")</f>
-        <v>m000008</v>
+      <c r="B9" s="7" t="s">
+        <v>168</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>154</v>
@@ -2078,9 +2155,8 @@
       <c r="A10" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="B10" s="7" t="str">
-        <f>"m00000" &amp; TEXT(ROW() - ROW(Table2[[#Headers],[UID]]), "0;-0")</f>
-        <v>m000009</v>
+      <c r="B10" s="7" t="s">
+        <v>184</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>180</v>
@@ -2100,6 +2176,60 @@
       <c r="J10" s="17"/>
       <c r="K10" s="8" t="s">
         <v>183</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="K11" s="8"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>202</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="H12" s="7"/>
+      <c r="I12" s="14" t="s">
+        <v>207</v>
+      </c>
+      <c r="J12" s="17"/>
+      <c r="K12" s="8" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -2117,7 +2247,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7750010-8426-4DA5-9D37-A1517A3A4563}">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
@@ -3027,6 +3157,123 @@
         <v>36</v>
       </c>
       <c r="C97" s="8"/>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B98" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="C98" s="8"/>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B99" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C99" s="8"/>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B100" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C100" s="8"/>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B101" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="C101" s="8"/>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B102" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="C102" s="8"/>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B103" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="C103" s="8"/>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B104" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="C104" s="8"/>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B105" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="C105" s="8"/>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B106" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="C106" s="8"/>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A107" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B107" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C107" s="8"/>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B108" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="C108" s="8"/>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B109" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="C109" s="8"/>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B110" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="C110" s="8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -3039,7 +3286,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7925662C-692A-4A45-AA4F-75A27046A9CD}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
@@ -3086,19 +3333,27 @@
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="8" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="8" t="s">
         <v>175</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -3111,7 +3366,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51CA61E6-D3C1-47E8-B2E1-3DBA27FAE247}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
@@ -3159,27 +3414,59 @@
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="8" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="8" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="8" t="s">
         <v>189</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>